<commit_message>
Emergency sync: backup all local changes due to bad computer
</commit_message>
<xml_diff>
--- a/dataAcquisition/Motec_MP/alias/driverAlias.xlsx
+++ b/dataAcquisition/Motec_MP/alias/driverAlias.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SimEnv\dataAcquisition\Motec_MP\alias\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A08856E-A2F2-499F-BB93-955AA8F57514}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{235D4B47-CDF5-4FC2-B925-F7B025E3DB7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1935" windowWidth="29040" windowHeight="15720" xr2:uid="{F4E9EF79-5CED-499A-8721-7FE03FA878BA}"/>
+    <workbookView xWindow="57480" yWindow="660" windowWidth="29040" windowHeight="15720" xr2:uid="{F4E9EF79-5CED-499A-8721-7FE03FA878BA}"/>
   </bookViews>
   <sheets>
     <sheet name="driverAlias" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="934" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="934" uniqueCount="250">
   <si>
     <t>Unique Drivers IDs</t>
   </si>
@@ -781,6 +781,9 @@
   </si>
   <si>
     <t>UKN</t>
+  </si>
+  <si>
+    <t>18-ADP</t>
   </si>
 </sst>
 </file>
@@ -3073,7 +3076,7 @@
         <v>154</v>
       </c>
       <c r="N14" t="s">
-        <v>117</v>
+        <v>249</v>
       </c>
       <c r="O14" t="s">
         <v>168</v>

</xml_diff>